<commit_message>
Update dataset preparation artifacts
</commit_message>
<xml_diff>
--- a/outputs/task5/task5_dataset_review.xlsx
+++ b/outputs/task5/task5_dataset_review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcbfaac0ba1e14594"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset Review" sheetId="2" r:id="Ra9732cfbf2184130"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graph Schema" sheetId="3" r:id="Ra7cbfd0b17dc40da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R7c32c2d7261f41cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R07d31b814cdb4c95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset Review" sheetId="2" r:id="R9dc81d45a0c04ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graph Schema" sheetId="3" r:id="R8eb78c8ab4ef4ec7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R7039dbd5ef28473c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -193,7 +193,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Summary'!$A$20:$A$25</c:f>
+              <c:f>'Summary'!$A$20:$A$27</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -201,7 +201,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Summary'!$B$20:$B$25</c:f>
+              <c:f>'Summary'!$B$20:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -217,7 +217,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Summary'!$A$20:$A$25</c:f>
+              <c:f>'Summary'!$A$20:$A$27</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -225,7 +225,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Summary'!$C$20:$C$25</c:f>
+              <c:f>'Summary'!$C$20:$C$27</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -241,7 +241,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'Summary'!$A$20:$A$25</c:f>
+              <c:f>'Summary'!$A$20:$A$27</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -249,7 +249,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Summary'!$D$20:$D$25</c:f>
+              <c:f>'Summary'!$D$20:$D$27</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="0"/>
@@ -364,7 +364,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R79ed010589ee4119"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6fc00fcc0b5a43b1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -374,7 +374,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Task5DatasetReview" displayName="Task5DatasetReview" ref="A1:V7" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Task5DatasetReview" displayName="Task5DatasetReview" ref="A1:V9" headerRowCount="1">
   <x:tableColumns count="22">
     <x:tableColumn id="1" name="dataset_id"/>
     <x:tableColumn id="2" name="name"/>
@@ -625,14 +625,14 @@
         <x:v>Candidate sources reviewed</x:v>
       </x:c>
       <x:c r="B4" s="31" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C4" s="19"/>
       <x:c r="D4" s="19" t="str">
         <x:v>core</x:v>
       </x:c>
       <x:c r="E4" s="19" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F4" s="19"/>
       <x:c r="G4" s="19"/>
@@ -649,7 +649,7 @@
         <x:v>Core datasets</x:v>
       </x:c>
       <x:c r="B5" s="31" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="19"/>
       <x:c r="D5" s="19" t="str">
@@ -813,10 +813,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>ReactionDataExtractor2</x:v>
+        <x:v>RxnCaption / U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
-        <x:v>Use as parser baseline and machine-readable graph output reference.</x:v>
+        <x:v>Add larger reaction-diagram topology, arrow and condition parsing coverage.</x:v>
       </x:c>
       <x:c r="D13" s="19" t="str"/>
       <x:c r="E13" s="19" t="str"/>
@@ -835,10 +835,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
-        <x:v>AI2D</x:v>
+        <x:v>ReactionDataExtractor2</x:v>
       </x:c>
       <x:c r="C14" s="19" t="str">
-        <x:v>Use only for generic diagram node-arrow-text transfer, with chemistry keyword filtering.</x:v>
+        <x:v>Use as parser baseline and machine-readable graph output reference.</x:v>
       </x:c>
       <x:c r="D14" s="19" t="str"/>
       <x:c r="E14" s="19" t="str"/>
@@ -857,10 +857,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>PIDCon</x:v>
+        <x:v>PID2Graph</x:v>
       </x:c>
       <x:c r="C15" s="19" t="str">
-        <x:v>Use for graph recovery evaluation with box-line-connection-path annotations.</x:v>
+        <x:v>Use as the core P&amp;ID graph-structure proxy for node-edge recovery.</x:v>
       </x:c>
       <x:c r="D15" s="19" t="str"/>
       <x:c r="E15" s="19" t="str"/>
@@ -879,10 +879,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B16" s="18" t="str">
-        <x:v>PID_dataset / Digitize-PID</x:v>
+        <x:v>PIDCon / PID_dataset / Digitize-PID</x:v>
       </x:c>
       <x:c r="C16" s="19" t="str">
-        <x:v>Use later for P&amp;ID/PFD extension after storage and license checks.</x:v>
+        <x:v>Use later for P&amp;ID/PFD extension after access, storage and license checks.</x:v>
       </x:c>
       <x:c r="D16" s="19" t="str"/>
       <x:c r="E16" s="19" t="str"/>
@@ -897,14 +897,20 @@
       <x:c r="N16" s="19"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="19"/>
-      <x:c r="B17" s="19"/>
-      <x:c r="C17" s="19"/>
-      <x:c r="D17" s="19"/>
-      <x:c r="E17" s="19"/>
-      <x:c r="F17" s="19"/>
-      <x:c r="G17" s="19"/>
-      <x:c r="H17" s="19"/>
+      <x:c r="A17" s="17" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B17" s="18" t="str">
+        <x:v>AI2D</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="str">
+        <x:v>Use only for generic diagram node-arrow-text transfer, with chemistry keyword filtering.</x:v>
+      </x:c>
+      <x:c r="D17" s="19" t="str"/>
+      <x:c r="E17" s="19" t="str"/>
+      <x:c r="F17" s="19" t="str"/>
+      <x:c r="G17" s="19" t="str"/>
+      <x:c r="H17" s="19" t="str"/>
       <x:c r="I17" s="19"/>
       <x:c r="J17" s="19"/>
       <x:c r="K17" s="19"/>
@@ -958,7 +964,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="19" t="str">
-        <x:v>PID_dataset</x:v>
+        <x:v>PID2Graph</x:v>
       </x:c>
       <x:c r="B20" s="19" t="n">
         <x:v>5</x:v>
@@ -970,10 +976,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E20" s="19" t="str">
-        <x:v>later_or_hold</x:v>
+        <x:v>core</x:v>
       </x:c>
       <x:c r="F20" s="19" t="str">
-        <x:v>Large archive and full P&amp;ID complexity may overwhelm a lightweight optional task.</x:v>
+        <x:v>P&amp;ID is an engineering proxy for PFD/process flow diagrams and may not contain reaction-r...</x:v>
       </x:c>
       <x:c r="G20" s="19"/>
       <x:c r="H20" s="19"/>
@@ -986,7 +992,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="19" t="str">
-        <x:v>PIDCon</x:v>
+        <x:v>PID_dataset</x:v>
       </x:c>
       <x:c r="B21" s="19" t="n">
         <x:v>5</x:v>
@@ -998,10 +1004,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E21" s="19" t="str">
-        <x:v>core</x:v>
+        <x:v>later_or_hold</x:v>
       </x:c>
       <x:c r="F21" s="19" t="str">
-        <x:v>More engineering-heavy than lightweight diagrams; download is via Baidu Disk and license ...</x:v>
+        <x:v>Large archive and full P&amp;ID complexity may overwhelm a lightweight optional task.</x:v>
       </x:c>
       <x:c r="G21" s="19"/>
       <x:c r="H21" s="19"/>
@@ -1014,22 +1020,22 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="19" t="str">
-        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
+        <x:v>PIDCon</x:v>
       </x:c>
       <x:c r="B22" s="19" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C22" s="19" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D22" s="19" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E22" s="19" t="str">
-        <x:v>auxiliary</x:v>
+        <x:v>core</x:v>
       </x:c>
       <x:c r="F22" s="19" t="str">
-        <x:v>Often symbol-only, so node-edge graph recovery may require added line/connectivity annota...</x:v>
+        <x:v>More engineering-heavy than lightweight diagrams; download is via Baidu Disk and license ...</x:v>
       </x:c>
       <x:c r="G22" s="19"/>
       <x:c r="H22" s="19"/>
@@ -1042,22 +1048,22 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="19" t="str">
-        <x:v>ReactionDataExtractor2</x:v>
+        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
       </x:c>
       <x:c r="B23" s="19" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C23" s="19" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E23" s="19" t="str">
         <x:v>auxiliary</x:v>
       </x:c>
       <x:c r="F23" s="19" t="str">
-        <x:v>Still reaction scheme oriented; dependency and model-weight setup is heavier than a pure ...</x:v>
+        <x:v>Often symbol-only, so node-edge graph recovery may require added line/connectivity annota...</x:v>
       </x:c>
       <x:c r="G23" s="19"/>
       <x:c r="H23" s="19"/>
@@ -1070,22 +1076,22 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="19" t="str">
-        <x:v>RxnScribe</x:v>
+        <x:v>RxnCaption / U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="B24" s="19" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C24" s="19" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D24" s="19" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E24" s="19" t="str">
         <x:v>core</x:v>
       </x:c>
       <x:c r="F24" s="19" t="str">
-        <x:v>Not an industrial PFD/P&amp;ID dataset; equipment such as pump, valve, vessel is mostly absen...</x:v>
+        <x:v>Reaction-diagram focused rather than industrial PFD/P&amp;ID; equipment nodes such as pump, v...</x:v>
       </x:c>
       <x:c r="G24" s="19"/>
       <x:c r="H24" s="19"/>
@@ -1098,22 +1104,22 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="19" t="str">
-        <x:v>AI2D</x:v>
+        <x:v>ReactionDataExtractor2</x:v>
       </x:c>
       <x:c r="B25" s="19" t="n">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D25" s="19" t="n">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E25" s="19" t="str">
-        <x:v>transfer_only</x:v>
+        <x:v>auxiliary</x:v>
       </x:c>
       <x:c r="F25" s="19" t="str">
-        <x:v>Not a chemical engineering dataset and lacks typical process equipment symbols.</x:v>
+        <x:v>Still reaction scheme oriented; dependency and model-weight setup is heavier than a pure ...</x:v>
       </x:c>
       <x:c r="G25" s="19"/>
       <x:c r="H25" s="19"/>
@@ -1125,12 +1131,24 @@
       <x:c r="N25" s="19"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="19"/>
-      <x:c r="B26" s="19"/>
-      <x:c r="C26" s="19"/>
-      <x:c r="D26" s="19"/>
-      <x:c r="E26" s="19"/>
-      <x:c r="F26" s="19"/>
+      <x:c r="A26" s="19" t="str">
+        <x:v>RxnScribe</x:v>
+      </x:c>
+      <x:c r="B26" s="19" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C26" s="19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D26" s="19" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E26" s="19" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="F26" s="19" t="str">
+        <x:v>Not an industrial PFD/P&amp;ID dataset; equipment such as pump, valve, vessel is mostly absen...</x:v>
+      </x:c>
       <x:c r="G26" s="19"/>
       <x:c r="H26" s="19"/>
       <x:c r="I26" s="19"/>
@@ -1141,12 +1159,24 @@
       <x:c r="N26" s="19"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="19"/>
-      <x:c r="B27" s="19"/>
-      <x:c r="C27" s="19"/>
-      <x:c r="D27" s="19"/>
-      <x:c r="E27" s="19"/>
-      <x:c r="F27" s="19"/>
+      <x:c r="A27" s="19" t="str">
+        <x:v>AI2D</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D27" s="19" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E27" s="19" t="str">
+        <x:v>transfer_only</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>Not a chemical engineering dataset and lacks typical process equipment symbols.</x:v>
+      </x:c>
       <x:c r="G27" s="19"/>
       <x:c r="H27" s="19"/>
       <x:c r="I27" s="19"/>
@@ -1245,9 +1275,10 @@
     <x:mergeCell ref="C14:H14"/>
     <x:mergeCell ref="C15:H15"/>
     <x:mergeCell ref="C16:H16"/>
+    <x:mergeCell ref="C17:H17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5f00ea5e224dbf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7b4bbc688714916"/>
 </x:worksheet>
 </file>
 
@@ -1349,19 +1380,19 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="19" t="str">
-        <x:v>pid_dataset</x:v>
+        <x:v>pid2graph</x:v>
       </x:c>
       <x:c r="B2" s="19" t="str">
-        <x:v>PID_dataset</x:v>
+        <x:v>PID2Graph</x:v>
       </x:c>
       <x:c r="C2" s="19" t="str">
-        <x:v>later_or_hold</x:v>
+        <x:v>core</x:v>
       </x:c>
       <x:c r="D2" s="19" t="str">
-        <x:v>keep_later_large_scale</x:v>
+        <x:v>keep_core_for_graph_eval</x:v>
       </x:c>
       <x:c r="E2" s="19" t="str">
-        <x:v>industrial_piping_and_instrumentation_drawings</x:v>
+        <x:v>pid_graph_structure_dataset</x:v>
       </x:c>
       <x:c r="F2" s="19" t="str">
         <x:v>missing</x:v>
@@ -1388,48 +1419,48 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N2" s="19" t="str">
-        <x:v>industrial_pfd_pid_symbol_detection_reference</x:v>
+        <x:v>core_pid_graph_structure_extraction</x:v>
       </x:c>
       <x:c r="O2" s="19" t="str">
-        <x:v>P&amp;ID images plus code/weights according to record; inspect archive for exact labels before model training</x:v>
+        <x:v>Symbols as graph nodes with bbox coordinates (xmin, ymin, xmax, ymax) and label; lines represent graph edges or symbol connections</x:v>
       </x:c>
       <x:c r="P2" s="19" t="str">
-        <x:v>Keep equipment, valve, vessel, instrument, and pipeline samples after license/provenance review; downsample for light process diagram transfer.</x:v>
+        <x:v>Keep images with complete node bbox/label and edge graph annotations; convert symbols to equipment nodes, lines to edges, and preserve connection direction or undirected connectivity where direction is not annotated.</x:v>
       </x:c>
       <x:c r="Q2" s="19" t="str">
-        <x:v>Large archive and full P&amp;ID complexity may overwhelm a lightweight optional task.</x:v>
+        <x:v>P&amp;ID is an engineering proxy for PFD/process flow diagrams and may not contain reaction-route chemistry conditions.</x:v>
       </x:c>
       <x:c r="R2" s="19" t="str">
-        <x:v>CC BY 4.0</x:v>
+        <x:v>CC BY-SA 4.0 for referenced PID sources noted in Zenodo record; verify exact archive terms before redistribution</x:v>
       </x:c>
       <x:c r="S2" s="19" t="str">
-        <x:v>https://zenodo.org/records/8028570</x:v>
+        <x:v>https://zenodo.org/records/14803338</x:v>
       </x:c>
       <x:c r="T2" s="19" t="str">
-        <x:v>https://zenodo.org/records/8028570</x:v>
+        <x:v>https://zenodo.org/records/14803338</x:v>
       </x:c>
       <x:c r="U2" s="19" t="str">
-        <x:v>Local dataset root not found; place files under data/raw/PID_dataset and rerun this audit.</x:v>
+        <x:v>Local dataset root not found; place files under data/raw/PID2Graph and rerun this audit.</x:v>
       </x:c>
       <x:c r="V2" s="19" t="str">
-        <x:v>Do not download by default; first reserve storage, download checksum-verified archive, then sample 50 drawings for symbol taxonomy mapping.</x:v>
+        <x:v>Download from Zenodo, checksum archives, inspect complete-plan graph files, then convert a 20-image sample into task5_graph_schema.json for validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="19" t="str">
-        <x:v>pidcon</x:v>
+        <x:v>pid_dataset</x:v>
       </x:c>
       <x:c r="B3" s="19" t="str">
-        <x:v>PIDCon</x:v>
+        <x:v>PID_dataset</x:v>
       </x:c>
       <x:c r="C3" s="19" t="str">
-        <x:v>core</x:v>
+        <x:v>later_or_hold</x:v>
       </x:c>
       <x:c r="D3" s="19" t="str">
-        <x:v>keep_core_for_graph_eval</x:v>
+        <x:v>keep_later_large_scale</x:v>
       </x:c>
       <x:c r="E3" s="19" t="str">
-        <x:v>pid_connectivity_graph_dataset</x:v>
+        <x:v>industrial_piping_and_instrumentation_drawings</x:v>
       </x:c>
       <x:c r="F3" s="19" t="str">
         <x:v>missing</x:v>
@@ -1456,48 +1487,48 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N3" s="19" t="str">
-        <x:v>graph_recovery_evaluation_and_connectivity_transfer</x:v>
+        <x:v>industrial_pfd_pid_symbol_detection_reference</x:v>
       </x:c>
       <x:c r="O3" s="19" t="str">
-        <x:v>Box (xywh,class), Line (xyxy,id), Connection [obj_1,obj_2], Path {line_1,...,line_n}</x:v>
+        <x:v>P&amp;ID images plus code/weights according to record; inspect archive for exact labels before model training</x:v>
       </x:c>
       <x:c r="P3" s="19" t="str">
-        <x:v>Keep all accessible images with box-line-connection-path annotations; convert directly to node-edge graph and evaluate GED/NCA.</x:v>
+        <x:v>Keep equipment, valve, vessel, instrument, and pipeline samples after license/provenance review; downsample for light process diagram transfer.</x:v>
       </x:c>
       <x:c r="Q3" s="19" t="str">
-        <x:v>More engineering-heavy than lightweight diagrams; download is via Baidu Disk and license is unclear.</x:v>
+        <x:v>Large archive and full P&amp;ID complexity may overwhelm a lightweight optional task.</x:v>
       </x:c>
       <x:c r="R3" s="19" t="str">
-        <x:v>No explicit repository license found as of audit; confirm before redistribution</x:v>
+        <x:v>CC BY 4.0</x:v>
       </x:c>
       <x:c r="S3" s="19" t="str">
-        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
+        <x:v>https://zenodo.org/records/8028570</x:v>
       </x:c>
       <x:c r="T3" s="19" t="str">
-        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
+        <x:v>https://zenodo.org/records/8028570</x:v>
       </x:c>
       <x:c r="U3" s="19" t="str">
-        <x:v>Local dataset root not found; place files under data/raw/PIDCon and rerun this audit.</x:v>
+        <x:v>Local dataset root not found; place files under data/raw/PID_dataset and rerun this audit.</x:v>
       </x:c>
       <x:c r="V3" s="19" t="str">
-        <x:v>Confirm access and license; normalize boxes, lines, connections, and paths into task5_graph_schema.json.</x:v>
+        <x:v>Do not download by default; first reserve storage, download checksum-verified archive, then sample 50 drawings for symbol taxonomy mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="19" t="str">
-        <x:v>digitize_pid</x:v>
+        <x:v>pidcon</x:v>
       </x:c>
       <x:c r="B4" s="19" t="str">
-        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
+        <x:v>PIDCon</x:v>
       </x:c>
       <x:c r="C4" s="19" t="str">
-        <x:v>auxiliary</x:v>
+        <x:v>core</x:v>
       </x:c>
       <x:c r="D4" s="19" t="str">
-        <x:v>keep_auxiliary_with_license_check</x:v>
+        <x:v>keep_core_for_graph_eval</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>synthetic_piping_and_instrumentation_drawings</x:v>
+        <x:v>pid_connectivity_graph_dataset</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
         <x:v>missing</x:v>
@@ -1518,54 +1549,54 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L4" s="19" t="str">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M4" s="19" t="str">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="N4" s="19" t="str">
-        <x:v>synthetic_symbol_detection_pretraining</x:v>
+        <x:v>graph_recovery_evaluation_and_connectivity_transfer</x:v>
       </x:c>
       <x:c r="O4" s="19" t="str">
-        <x:v>Object detection style symbol labels; public mirrors often provide YOLO or imagefolder variants</x:v>
+        <x:v>Box (xywh,class), Line (xyxy,id), Connection [obj_1,obj_2], Path {line_1,...,line_n}</x:v>
       </x:c>
       <x:c r="P4" s="19" t="str">
-        <x:v>Keep synthetic P&amp;ID images with symbol boxes; map symbols to task equipment nodes and infer line/edge data only if annotation is present.</x:v>
+        <x:v>Keep all accessible images with box-line-connection-path annotations; convert directly to node-edge graph and evaluate GED/NCA.</x:v>
       </x:c>
       <x:c r="Q4" s="19" t="str">
-        <x:v>Often symbol-only, so node-edge graph recovery may require added line/connectivity annotation.</x:v>
+        <x:v>More engineering-heavy than lightweight diagrams; download is via Baidu Disk and license is unclear.</x:v>
       </x:c>
       <x:c r="R4" s="19" t="str">
-        <x:v>Original Google Drive terms need verification; derived Hugging Face mirrors vary</x:v>
+        <x:v>No explicit repository license found as of audit; confirm before redistribution</x:v>
       </x:c>
       <x:c r="S4" s="19" t="str">
-        <x:v>https://arxiv.org/abs/2109.03794</x:v>
+        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
       </x:c>
       <x:c r="T4" s="19" t="str">
-        <x:v>https://drive.google.com/drive/u/1/folders/1gMm_YKBZtXB3qUKUpI-LF1HE_MgzwfeR</x:v>
+        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
       </x:c>
       <x:c r="U4" s="19" t="str">
-        <x:v>Local dataset root not found; place files under data/raw/Dataset-PID and rerun this audit.</x:v>
+        <x:v>Local dataset root not found; place files under data/raw/PIDCon and rerun this audit.</x:v>
       </x:c>
       <x:c r="V4" s="19" t="str">
-        <x:v>Prefer original Drive or a documented Hugging Face mirror; verify symbol class list and train/val split before ingestion.</x:v>
+        <x:v>Confirm access and license; normalize boxes, lines, connections, and paths into task5_graph_schema.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="19" t="str">
-        <x:v>rde2</x:v>
+        <x:v>digitize_pid</x:v>
       </x:c>
       <x:c r="B5" s="19" t="str">
-        <x:v>ReactionDataExtractor2</x:v>
+        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
         <x:v>auxiliary</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>keep_auxiliary</x:v>
+        <x:v>keep_auxiliary_with_license_check</x:v>
       </x:c>
       <x:c r="E5" s="19" t="str">
-        <x:v>chemical_reaction_scheme_toolkit</x:v>
+        <x:v>synthetic_piping_and_instrumentation_drawings</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
         <x:v>missing</x:v>
@@ -1586,45 +1617,45 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L5" s="19" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M5" s="19" t="str">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="N5" s="19" t="str">
-        <x:v>baseline_parser_and_schema_reference</x:v>
+        <x:v>synthetic_symbol_detection_pretraining</x:v>
       </x:c>
       <x:c r="O5" s="19" t="str">
-        <x:v>Detected nodes and adjacency dictionary for reaction scheme entities; arrows, conditions, diagrams, labels</x:v>
+        <x:v>Object detection style symbol labels; public mirrors often provide YOLO or imagefolder variants</x:v>
       </x:c>
       <x:c r="P5" s="19" t="str">
-        <x:v>Use as a baseline and schema normalizer; keep only outputs generated from chemical reaction scheme images with valid node list and adjacency dictionary.</x:v>
+        <x:v>Keep synthetic P&amp;ID images with symbol boxes; map symbols to task equipment nodes and infer line/edge data only if annotation is present.</x:v>
       </x:c>
       <x:c r="Q5" s="19" t="str">
-        <x:v>Still reaction scheme oriented; dependency and model-weight setup is heavier than a pure dataset.</x:v>
+        <x:v>Often symbol-only, so node-edge graph recovery may require added line/connectivity annotation.</x:v>
       </x:c>
       <x:c r="R5" s="19" t="str">
-        <x:v>MIT</x:v>
+        <x:v>Original Google Drive terms need verification; derived Hugging Face mirrors vary</x:v>
       </x:c>
       <x:c r="S5" s="19" t="str">
-        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+        <x:v>https://arxiv.org/abs/2109.03794</x:v>
       </x:c>
       <x:c r="T5" s="19" t="str">
-        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+        <x:v>https://drive.google.com/drive/u/1/folders/1gMm_YKBZtXB3qUKUpI-LF1HE_MgzwfeR</x:v>
       </x:c>
       <x:c r="U5" s="19" t="str">
-        <x:v>Local dataset root not found; place files under data/raw/ReactionDataExtractor2 and rerun this audit.</x:v>
+        <x:v>Local dataset root not found; place files under data/raw/Dataset-PID and rerun this audit.</x:v>
       </x:c>
       <x:c r="V5" s="19" t="str">
-        <x:v>Install in isolated environment if needed; run on a small RxnScribe/own sample batch and normalize outputs to task5_graph_schema.json.</x:v>
+        <x:v>Prefer original Drive or a documented Hugging Face mirror; verify symbol class list and train/val split before ingestion.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="19" t="str">
-        <x:v>rxnscribe</x:v>
+        <x:v>urxndiagram15k</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
-        <x:v>RxnScribe</x:v>
+        <x:v>RxnCaption / U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
         <x:v>core</x:v>
@@ -1633,7 +1664,7 @@
         <x:v>keep_core</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>chemical_reaction_scheme</x:v>
+        <x:v>chemical_reaction_diagram_parsing</x:v>
       </x:c>
       <x:c r="F6" s="19" t="str">
         <x:v>missing</x:v>
@@ -1654,54 +1685,54 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="L6" s="19" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M6" s="19" t="str">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="N6" s="19" t="str">
-        <x:v>core_reaction_scheme_graph_pretraining</x:v>
+        <x:v>large_reaction_diagram_node_arrow_condition_training</x:v>
       </x:c>
       <x:c r="O6" s="19" t="str">
-        <x:v>reactants, conditions, products with bounding boxes, OCR text, SMILES/molfile when recognized</x:v>
+        <x:v>Reaction diagram images with detailed annotations for parsing reaction entities, arrows, conditions and topology structure</x:v>
       </x:c>
       <x:c r="P6" s="19" t="str">
-        <x:v>Keep reaction diagrams with complete image and ground-truth split records; map reactants/products to nodes, reaction arrows to directed edges, and conditions text to parameters.</x:v>
+        <x:v>Keep samples with valid image paths and ground_truth annotations; map molecule/reagent/condition regions to nodes or parameters, reaction arrows to directed edges, and topology class to graph metadata.</x:v>
       </x:c>
       <x:c r="Q6" s="19" t="str">
-        <x:v>Not an industrial PFD/P&amp;ID dataset; equipment such as pump, valve, vessel is mostly absent.</x:v>
+        <x:v>Reaction-diagram focused rather than industrial PFD/P&amp;ID; equipment nodes such as pump, valve, heat exchanger and vessel are not the main target.</x:v>
       </x:c>
       <x:c r="R6" s="19" t="str">
-        <x:v>MIT for code repository; verify dataset/model terms on Hugging Face before redistribution</x:v>
+        <x:v>Verify Hugging Face dataset card and upstream paper terms before redistribution</x:v>
       </x:c>
       <x:c r="S6" s="19" t="str">
-        <x:v>https://github.com/thomas0809/RxnScribe</x:v>
+        <x:v>https://huggingface.co/datasets/songjhPKU/U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="T6" s="19" t="str">
-        <x:v>https://huggingface.co/yujieq/RxnScribe/blob/main/images.zip</x:v>
+        <x:v>https://huggingface.co/datasets/songjhPKU/U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="U6" s="19" t="str">
-        <x:v>Local dataset root not found; place files under data/raw/RxnScribe and rerun this audit.</x:v>
+        <x:v>Local dataset root not found; place files under data/raw/U-RxnDiagram-15k and rerun this audit.</x:v>
       </x:c>
       <x:c r="V6" s="19" t="str">
-        <x:v>Download images.zip only when storage permits; parse data/parse/splits into graph JSONL; audit OCR condition quality.</x:v>
+        <x:v>Download through Hugging Face when storage and license review are ready; validate train/test image counts, annotation JSON schema and topology labels before conversion.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="19" t="str">
-        <x:v>ai2d</x:v>
+        <x:v>rde2</x:v>
       </x:c>
       <x:c r="B7" s="19" t="str">
-        <x:v>AI2D</x:v>
+        <x:v>ReactionDataExtractor2</x:v>
       </x:c>
       <x:c r="C7" s="19" t="str">
-        <x:v>transfer_only</x:v>
+        <x:v>auxiliary</x:v>
       </x:c>
       <x:c r="D7" s="19" t="str">
-        <x:v>keep_transfer_only</x:v>
+        <x:v>keep_auxiliary</x:v>
       </x:c>
       <x:c r="E7" s="19" t="str">
-        <x:v>general_science_diagram</x:v>
+        <x:v>chemical_reaction_scheme_toolkit</x:v>
       </x:c>
       <x:c r="F7" s="19" t="str">
         <x:v>missing</x:v>
@@ -1719,46 +1750,182 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="19" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L7" s="19" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M7" s="19" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N7" s="19" t="str">
+        <x:v>baseline_parser_and_schema_reference</x:v>
+      </x:c>
+      <x:c r="O7" s="19" t="str">
+        <x:v>Detected nodes and adjacency dictionary for reaction scheme entities; arrows, conditions, diagrams, labels</x:v>
+      </x:c>
+      <x:c r="P7" s="19" t="str">
+        <x:v>Use as a baseline and schema normalizer; keep only outputs generated from chemical reaction scheme images with valid node list and adjacency dictionary.</x:v>
+      </x:c>
+      <x:c r="Q7" s="19" t="str">
+        <x:v>Still reaction scheme oriented; dependency and model-weight setup is heavier than a pure dataset.</x:v>
+      </x:c>
+      <x:c r="R7" s="19" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="S7" s="19" t="str">
+        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+      </x:c>
+      <x:c r="T7" s="19" t="str">
+        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+      </x:c>
+      <x:c r="U7" s="19" t="str">
+        <x:v>Local dataset root not found; place files under data/raw/ReactionDataExtractor2 and rerun this audit.</x:v>
+      </x:c>
+      <x:c r="V7" s="19" t="str">
+        <x:v>Install in isolated environment if needed; run on a small RxnScribe/own sample batch and normalize outputs to task5_graph_schema.json.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="19" t="str">
+        <x:v>rxnscribe</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>RxnScribe</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>keep_core</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>chemical_reaction_scheme</x:v>
+      </x:c>
+      <x:c r="F8" s="19" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="G8" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="19" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="L8" s="19" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M8" s="19" t="str">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N8" s="19" t="str">
+        <x:v>core_reaction_scheme_graph_pretraining</x:v>
+      </x:c>
+      <x:c r="O8" s="19" t="str">
+        <x:v>reactants, conditions, products with bounding boxes, OCR text, SMILES/molfile when recognized</x:v>
+      </x:c>
+      <x:c r="P8" s="19" t="str">
+        <x:v>Keep reaction diagrams with complete image and ground-truth split records; map reactants/products to nodes, reaction arrows to directed edges, and conditions text to parameters.</x:v>
+      </x:c>
+      <x:c r="Q8" s="19" t="str">
+        <x:v>Not an industrial PFD/P&amp;ID dataset; equipment such as pump, valve, vessel is mostly absent.</x:v>
+      </x:c>
+      <x:c r="R8" s="19" t="str">
+        <x:v>MIT for code repository; verify dataset/model terms on Hugging Face before redistribution</x:v>
+      </x:c>
+      <x:c r="S8" s="19" t="str">
+        <x:v>https://github.com/thomas0809/RxnScribe</x:v>
+      </x:c>
+      <x:c r="T8" s="19" t="str">
+        <x:v>https://huggingface.co/yujieq/RxnScribe/blob/main/images.zip</x:v>
+      </x:c>
+      <x:c r="U8" s="19" t="str">
+        <x:v>Local dataset root not found; place files under data/raw/RxnScribe and rerun this audit.</x:v>
+      </x:c>
+      <x:c r="V8" s="19" t="str">
+        <x:v>Download images.zip only when storage permits; parse data/parse/splits into graph JSONL; audit OCR condition quality.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="19" t="str">
+        <x:v>ai2d</x:v>
+      </x:c>
+      <x:c r="B9" s="19" t="str">
+        <x:v>AI2D</x:v>
+      </x:c>
+      <x:c r="C9" s="19" t="str">
+        <x:v>transfer_only</x:v>
+      </x:c>
+      <x:c r="D9" s="19" t="str">
+        <x:v>keep_transfer_only</x:v>
+      </x:c>
+      <x:c r="E9" s="19" t="str">
+        <x:v>general_science_diagram</x:v>
+      </x:c>
+      <x:c r="F9" s="19" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="G9" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="19" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K9" s="19" t="str">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="L7" s="19" t="str">
+      <x:c r="L9" s="19" t="str">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="M7" s="19" t="str">
+      <x:c r="M9" s="19" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="N7" s="19" t="str">
+      <x:c r="N9" s="19" t="str">
         <x:v>generic_diagram_node_arrow_text_pretraining</x:v>
       </x:c>
-      <x:c r="O7" s="19" t="str">
+      <x:c r="O9" s="19" t="str">
         <x:v>Object segmentations, diagrammatic elements, text elements, question-answer annotations</x:v>
       </x:c>
-      <x:c r="P7" s="19" t="str">
+      <x:c r="P9" s="19" t="str">
         <x:v>Keep only samples whose labels/text indicate chemistry, process, flow, reaction, heat, gas, liquid, apparatus, or arrow-rich scientific diagrams; otherwise use as generic pretraining only.</x:v>
       </x:c>
-      <x:c r="Q7" s="19" t="str">
+      <x:c r="Q9" s="19" t="str">
         <x:v>Not a chemical engineering dataset and lacks typical process equipment symbols.</x:v>
       </x:c>
-      <x:c r="R7" s="19" t="str">
+      <x:c r="R9" s="19" t="str">
         <x:v>Check AI2D terms before redistribution; dataset is hosted by AllenAI</x:v>
       </x:c>
-      <x:c r="S7" s="19" t="str">
+      <x:c r="S9" s="19" t="str">
         <x:v>https://prior.allenai.org/projects/diagram-understanding</x:v>
       </x:c>
-      <x:c r="T7" s="19" t="str">
+      <x:c r="T9" s="19" t="str">
         <x:v>http://ai2-website.s3.amazonaws.com/data/ai2d-all.zip</x:v>
       </x:c>
-      <x:c r="U7" s="19" t="str">
+      <x:c r="U9" s="19" t="str">
         <x:v>Local dataset root not found; place files under data/raw/AI2D and rerun this audit.</x:v>
       </x:c>
-      <x:c r="V7" s="19" t="str">
+      <x:c r="V9" s="19" t="str">
         <x:v>After download, keyword-filter annotations/text; sample 100 diagrams to estimate chemistry subset size before full conversion.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a62c1c5971448db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R417de674ff6449e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2030,103 +2197,137 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="19" t="str">
-        <x:v>PID_dataset</x:v>
+        <x:v>PID2Graph</x:v>
       </x:c>
       <x:c r="B2" s="19" t="str">
-        <x:v>https://zenodo.org/records/8028570</x:v>
+        <x:v>https://zenodo.org/records/14803338</x:v>
       </x:c>
       <x:c r="C2" s="19" t="str">
-        <x:v>https://zenodo.org/records/8028570</x:v>
+        <x:v>https://zenodo.org/records/14803338</x:v>
       </x:c>
       <x:c r="D2" s="19" t="str">
-        <x:v>CC BY 4.0</x:v>
+        <x:v>CC BY-SA 4.0 for referenced PID sources noted in Zenodo record; verify exact archive terms before redistribution</x:v>
       </x:c>
       <x:c r="E2" s="19" t="str">
-        <x:v>Do not download by default; first reserve storage, download checksum-verified archive, then sample 50 drawings for symbol taxonomy mapping.</x:v>
+        <x:v>Download from Zenodo, checksum archives, inspect complete-plan graph files, then convert a 20-image sample into task5_graph_schema.json for validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="19" t="str">
-        <x:v>PIDCon</x:v>
+        <x:v>PID_dataset</x:v>
       </x:c>
       <x:c r="B3" s="19" t="str">
-        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
+        <x:v>https://zenodo.org/records/8028570</x:v>
       </x:c>
       <x:c r="C3" s="19" t="str">
-        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
+        <x:v>https://zenodo.org/records/8028570</x:v>
       </x:c>
       <x:c r="D3" s="19" t="str">
-        <x:v>No explicit repository license found as of audit; confirm before redistribution</x:v>
+        <x:v>CC BY 4.0</x:v>
       </x:c>
       <x:c r="E3" s="19" t="str">
-        <x:v>Confirm access and license; normalize boxes, lines, connections, and paths into task5_graph_schema.json.</x:v>
+        <x:v>Do not download by default; first reserve storage, download checksum-verified archive, then sample 50 drawings for symbol taxonomy mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="19" t="str">
-        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
+        <x:v>PIDCon</x:v>
       </x:c>
       <x:c r="B4" s="19" t="str">
-        <x:v>https://arxiv.org/abs/2109.03794</x:v>
+        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
       </x:c>
       <x:c r="C4" s="19" t="str">
-        <x:v>https://drive.google.com/drive/u/1/folders/1gMm_YKBZtXB3qUKUpI-LF1HE_MgzwfeR</x:v>
+        <x:v>https://github.com/sad123-yx/PIDCon</x:v>
       </x:c>
       <x:c r="D4" s="19" t="str">
-        <x:v>Original Google Drive terms need verification; derived Hugging Face mirrors vary</x:v>
+        <x:v>No explicit repository license found as of audit; confirm before redistribution</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>Prefer original Drive or a documented Hugging Face mirror; verify symbol class list and train/val split before ingestion.</x:v>
+        <x:v>Confirm access and license; normalize boxes, lines, connections, and paths into task5_graph_schema.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="19" t="str">
-        <x:v>ReactionDataExtractor2</x:v>
+        <x:v>Dataset-P&amp;ID / Digitize-PID</x:v>
       </x:c>
       <x:c r="B5" s="19" t="str">
-        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+        <x:v>https://arxiv.org/abs/2109.03794</x:v>
       </x:c>
       <x:c r="C5" s="19" t="str">
-        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+        <x:v>https://drive.google.com/drive/u/1/folders/1gMm_YKBZtXB3qUKUpI-LF1HE_MgzwfeR</x:v>
       </x:c>
       <x:c r="D5" s="19" t="str">
-        <x:v>MIT</x:v>
+        <x:v>Original Google Drive terms need verification; derived Hugging Face mirrors vary</x:v>
       </x:c>
       <x:c r="E5" s="19" t="str">
-        <x:v>Install in isolated environment if needed; run on a small RxnScribe/own sample batch and normalize outputs to task5_graph_schema.json.</x:v>
+        <x:v>Prefer original Drive or a documented Hugging Face mirror; verify symbol class list and train/val split before ingestion.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="19" t="str">
-        <x:v>RxnScribe</x:v>
+        <x:v>RxnCaption / U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="B6" s="19" t="str">
-        <x:v>https://github.com/thomas0809/RxnScribe</x:v>
+        <x:v>https://huggingface.co/datasets/songjhPKU/U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="C6" s="19" t="str">
-        <x:v>https://huggingface.co/yujieq/RxnScribe/blob/main/images.zip</x:v>
+        <x:v>https://huggingface.co/datasets/songjhPKU/U-RxnDiagram-15k</x:v>
       </x:c>
       <x:c r="D6" s="19" t="str">
-        <x:v>MIT for code repository; verify dataset/model terms on Hugging Face before redistribution</x:v>
+        <x:v>Verify Hugging Face dataset card and upstream paper terms before redistribution</x:v>
       </x:c>
       <x:c r="E6" s="19" t="str">
-        <x:v>Download images.zip only when storage permits; parse data/parse/splits into graph JSONL; audit OCR condition quality.</x:v>
+        <x:v>Download through Hugging Face when storage and license review are ready; validate train/test image counts, annotation JSON schema and topology labels before conversion.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="19" t="str">
+        <x:v>ReactionDataExtractor2</x:v>
+      </x:c>
+      <x:c r="B7" s="19" t="str">
+        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+      </x:c>
+      <x:c r="C7" s="19" t="str">
+        <x:v>https://github.com/dmw51/reactiondataextractor2</x:v>
+      </x:c>
+      <x:c r="D7" s="19" t="str">
+        <x:v>MIT</x:v>
+      </x:c>
+      <x:c r="E7" s="19" t="str">
+        <x:v>Install in isolated environment if needed; run on a small RxnScribe/own sample batch and normalize outputs to task5_graph_schema.json.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="19" t="str">
+        <x:v>RxnScribe</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
+        <x:v>https://github.com/thomas0809/RxnScribe</x:v>
+      </x:c>
+      <x:c r="C8" s="19" t="str">
+        <x:v>https://huggingface.co/yujieq/RxnScribe/blob/main/images.zip</x:v>
+      </x:c>
+      <x:c r="D8" s="19" t="str">
+        <x:v>MIT for code repository; verify dataset/model terms on Hugging Face before redistribution</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
+        <x:v>Download images.zip only when storage permits; parse data/parse/splits into graph JSONL; audit OCR condition quality.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="19" t="str">
         <x:v>AI2D</x:v>
       </x:c>
-      <x:c r="B7" s="19" t="str">
+      <x:c r="B9" s="19" t="str">
         <x:v>https://prior.allenai.org/projects/diagram-understanding</x:v>
       </x:c>
-      <x:c r="C7" s="19" t="str">
+      <x:c r="C9" s="19" t="str">
         <x:v>http://ai2-website.s3.amazonaws.com/data/ai2d-all.zip</x:v>
       </x:c>
-      <x:c r="D7" s="19" t="str">
+      <x:c r="D9" s="19" t="str">
         <x:v>Check AI2D terms before redistribution; dataset is hosted by AllenAI</x:v>
       </x:c>
-      <x:c r="E7" s="19" t="str">
+      <x:c r="E9" s="19" t="str">
         <x:v>After download, keyword-filter annotations/text; sample 100 diagrams to estimate chemistry subset size before full conversion.</x:v>
       </x:c>
     </x:row>

</xml_diff>